<commit_message>
Rename RORPractitionerProfile/RORPractitionerRoleProfile to RORPractitioner/RORPractitionerRole
Drops the "Profile" suffix now that the old RORPractitioner/RORPractitionerRole
names are free (renamed to RORPerson / split apart in the previous commit).
Updates cross-references in RORPerson, RORTask, RORMeasureReport and the
impact analysis doc accordingly.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com> 7beb0a137da49baee2343bebd1fd9632b0fc2750
</commit_message>
<xml_diff>
--- a/update-dependencies-fr-core-annuaire/ig/StructureDefinition-ror-person.xlsx
+++ b/update-dependencies-fr-core-annuaire/ig/StructureDefinition-ror-person.xlsx
@@ -57,7 +57,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-21T09:28:33+00:00</t>
+    <t>2026-08-21T09:39:43+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -1355,7 +1355,7 @@
     <t>as-practitioner-exercice-professionnel</t>
   </si>
   <si>
-    <t>Référence vers l'exercice professionnel (RORPractitionerProfile) de la personne</t>
+    <t>Référence vers l'exercice professionnel (RORPractitioner) de la personne</t>
   </si>
   <si>
     <t>Person.link:as-practitioner-exercice-professionnel.id</t>

</xml_diff>